<commit_message>
feat: modulo de permisos dinamicos RBAC, rediseno responsive de Login CESMAG y limpieza de scripts
</commit_message>
<xml_diff>
--- a/frontend/public/plantilla_docentes_SIGAP.xlsx
+++ b/frontend/public/plantilla_docentes_SIGAP.xlsx
@@ -4,14 +4,15 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Plantilla Importación Usuarios" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Importar Usuarios" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Guía y Ejemplos" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="44">
   <si>
     <r>
       <rPr>
@@ -30,7 +31,7 @@
         <sz val="11"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">SISTEMA INTEGRADO DE GESTIÓN ACADÉMICA (SIGAP)
+      <t xml:space="preserve">SISTEMA INTEGRADO DE GESTIÓN ACADÉMICA PROFESORAL (SIGAP)
 </t>
     </r>
     <r>
@@ -44,7 +45,7 @@
     </r>
   </si>
   <si>
-    <t>📌 INSTRUCCIONES: Los campos marcados con (*) son obligatorios. En "Roles" puede especificar uno o varios roles separados por coma (ej. Docente, Director). Para usuarios que sean solo Consultor o Planeación, la columna "Programa Académico" puede quedar como "No aplica".</t>
+    <t>📌 INSTRUCCIONES: Diligencie sus datos a partir de la fila 10. La fila 9 es una fila de marca de agua/guía informativa. Los campos con (*) son obligatorios. Para múltiples roles sepárelos por coma (ej. Docente, Director). Para Consultor o Planeación sin programa use "No aplica". Consulte la hoja "Guía y Ejemplos" para más detalles.</t>
   </si>
   <si>
     <t>Nombres *</t>
@@ -68,101 +69,116 @@
     <t>Programa Académico</t>
   </si>
   <si>
-    <t>Juan Carlos</t>
-  </si>
-  <si>
-    <t>Pérez Gómez</t>
+    <t>Ej: Juan Carlos</t>
+  </si>
+  <si>
+    <t>Ej: Pérez Gómez</t>
   </si>
   <si>
     <t>CC</t>
   </si>
   <si>
-    <t>1085123456</t>
-  </si>
-  <si>
-    <t>jperez@cesmag.edu.co</t>
-  </si>
-  <si>
-    <t>Docente</t>
-  </si>
-  <si>
-    <t>Ingeniería de Sistemas</t>
-  </si>
-  <si>
-    <t>María Elena</t>
-  </si>
-  <si>
-    <t>Rodríguez López</t>
-  </si>
-  <si>
-    <t>1085987654</t>
-  </si>
-  <si>
-    <t>mrodriguez@cesmag.edu.co</t>
-  </si>
-  <si>
-    <t>Docente, Director</t>
-  </si>
-  <si>
-    <t>Ingeniería Electrónica</t>
-  </si>
-  <si>
-    <t>Carlos Andrés</t>
-  </si>
-  <si>
-    <t>Benavides Rosero</t>
-  </si>
-  <si>
-    <t>1085112233</t>
-  </si>
-  <si>
-    <t>cbenavides@cesmag.edu.co</t>
-  </si>
-  <si>
-    <t>Consultor, Planeación</t>
-  </si>
-  <si>
-    <t>No aplica</t>
-  </si>
-  <si>
-    <t>Ana Milena</t>
-  </si>
-  <si>
-    <t>Torres Burbano</t>
-  </si>
-  <si>
-    <t>1085445566</t>
-  </si>
-  <si>
-    <t>atorres@cesmag.edu.co</t>
-  </si>
-  <si>
-    <t>Ingeniería Industrial</t>
-  </si>
-  <si>
-    <t>Luis Fernando</t>
-  </si>
-  <si>
-    <t>Díaz Salazar</t>
-  </si>
-  <si>
-    <t>CE</t>
-  </si>
-  <si>
-    <t>1085778899</t>
-  </si>
-  <si>
-    <t>ldiaz@cesmag.edu.co</t>
-  </si>
-  <si>
-    <t>Director</t>
+    <t>Ej: 1085123456</t>
+  </si>
+  <si>
+    <t>Ej: jperez@cesmag.edu.co</t>
+  </si>
+  <si>
+    <t>Ej: Docente, Director</t>
+  </si>
+  <si>
+    <t>Ej: Ingeniería de Sistemas</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>GUÍA OFICIAL DE DILIGENCIAMIENTO - IMPORTACIÓN MASIVA SIGAP</t>
+  </si>
+  <si>
+    <t>Campo</t>
+  </si>
+  <si>
+    <t>Obligatorio</t>
+  </si>
+  <si>
+    <t>Valores Permitidos / Formato</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>Nombres</t>
+  </si>
+  <si>
+    <t>SÍ</t>
+  </si>
+  <si>
+    <t>Texto (ej. Juan Carlos)</t>
+  </si>
+  <si>
+    <t>Primer y segundo nombre del usuario.</t>
+  </si>
+  <si>
+    <t>Apellidos</t>
+  </si>
+  <si>
+    <t>Texto (ej. Pérez Gómez)</t>
+  </si>
+  <si>
+    <t>Primer y segundo apellido del usuario.</t>
+  </si>
+  <si>
+    <t>Tipo Documento</t>
+  </si>
+  <si>
+    <t>CC, CE, TI, Pasaporte</t>
+  </si>
+  <si>
+    <t>Tipo de documento de identificación oficial.</t>
+  </si>
+  <si>
+    <t>Número Documento</t>
+  </si>
+  <si>
+    <t>Numérico (ej. 1085123456)</t>
+  </si>
+  <si>
+    <t>Debe ser único en el sistema.</t>
+  </si>
+  <si>
+    <t>Correo Institucional</t>
+  </si>
+  <si>
+    <t>usuario@cesmag.edu.co</t>
+  </si>
+  <si>
+    <t>Correo válido institucional con dominio CESMAG.</t>
+  </si>
+  <si>
+    <t>Roles</t>
+  </si>
+  <si>
+    <t>Docente, Director, Consultor, Planeación</t>
+  </si>
+  <si>
+    <t>Puede ingresar uno o varios separados por coma.</t>
+  </si>
+  <si>
+    <t>Condicional</t>
+  </si>
+  <si>
+    <t>Ingeniería de Sistemas, Electrónica, Industrial, Financiera...</t>
+  </si>
+  <si>
+    <t>Requerido para Docente y Director. Si es solo Consultor o Planeación use "No aplica".</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -178,6 +194,25 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF94A3B8"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <color rgb="FF1E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -185,7 +220,7 @@
       <sz val="9.5"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -195,6 +230,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1A2744"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -209,11 +249,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
+        <fgColor rgb="FF334155"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -238,6 +278,21 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="dashed">
+        <color rgb="FF94A3B8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FFE2E8F0"/>
       </left>
       <right style="thin">
@@ -255,7 +310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -272,11 +327,35 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -300,13 +379,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>24000</xdr:colOff>
+      <xdr:colOff>39000</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>36000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>215999</xdr:colOff>
+      <xdr:colOff>221000</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>143999</xdr:rowOff>
     </xdr:to>
@@ -666,15 +745,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="34" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
-    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="1" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.25">
@@ -708,7 +787,7 @@
       <c r="G4" s="1"/>
     </row>
     <row r="5" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="6" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
@@ -720,7 +799,7 @@
       <c r="G6" s="2"/>
     </row>
     <row r="7" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>2</v>
       </c>
@@ -743,7 +822,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>9</v>
       </c>
@@ -766,96 +845,602 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>16</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>32</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -863,8 +1448,159 @@
     <mergeCell ref="C1:G4"/>
     <mergeCell ref="A6:G6"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="C10:C35">
+      <formula1>"CC,CE,TI,Pasaporte"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>